<commit_message>
Fix CA gap values and use product_code for bonds in ir_gap_beh_a
Three bugs fixed:
1. load_ir_gap_ca() now reads from irrbb.ir_gap_beh_a (product_name='6000')
   instead of deposit_beh, so gap_cf formula (capital+int) and tenor bucket
   dates match ir_gap_beh exactly.
2. Merge in compute_nii now includes bs_side to avoid double-counting the CA
   gap when both A-side and L-side rows share the same (currency, cf_end_dt).
3. Added product_code to sched.fin_inst (dict_tbl_sched_id_cols) and updated
   fin_inst_beh_a_q to use product_code instead of rate_type, so bonds show
   3000/3100 instead of F/V in ir_gap_beh_a.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/irrbb_calc/output/nii_results.xlsx
+++ b/irrbb_calc/output/nii_results.xlsx
@@ -506,25 +506,25 @@
         <v>0.9972602739726028</v>
       </c>
       <c r="E2" t="n">
-        <v>-5999621555.39</v>
+        <v>-11969286612.3</v>
       </c>
       <c r="F2" t="n">
-        <v>-8000000000</v>
+        <v>-8011508504.57</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>-59831842.36060165</v>
+        <v>-119364940.4623891</v>
       </c>
       <c r="I2" t="n">
-        <v>-19948979.55720657</v>
+        <v>39469348.8003759</v>
       </c>
       <c r="J2" t="n">
-        <v>-59831842.36060165</v>
+        <v>-119364940.4623891</v>
       </c>
       <c r="K2" t="n">
-        <v>-19948979.55720657</v>
+        <v>39469348.8003759</v>
       </c>
     </row>
     <row r="3">
@@ -545,25 +545,25 @@
         <v>0.9166666666666666</v>
       </c>
       <c r="E3" t="n">
-        <v>2175377097.22</v>
+        <v>4214343154.54</v>
       </c>
       <c r="F3" t="n">
-        <v>-400000000</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>19940956.72451666</v>
+        <v>38631478.91661666</v>
       </c>
       <c r="I3" t="n">
-        <v>-23607623.39118333</v>
+        <v>-38631478.91661666</v>
       </c>
       <c r="J3" t="n">
-        <v>19940956.72451666</v>
+        <v>38631478.91661666</v>
       </c>
       <c r="K3" t="n">
-        <v>-23607623.39118333</v>
+        <v>-38631478.91661666</v>
       </c>
     </row>
     <row r="4">
@@ -584,25 +584,25 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="E4" t="n">
-        <v>10750880995.23</v>
+        <v>21654457449.59</v>
       </c>
       <c r="F4" t="n">
-        <v>-800000000</v>
+        <v>-1888284222.06</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>89590674.96025001</v>
+        <v>180453812.0799167</v>
       </c>
       <c r="I4" t="n">
-        <v>-96257341.62691666</v>
+        <v>-196189513.9304167</v>
       </c>
       <c r="J4" t="n">
-        <v>89590674.96025001</v>
+        <v>180453812.0799167</v>
       </c>
       <c r="K4" t="n">
-        <v>-96257341.62691666</v>
+        <v>-196189513.9304167</v>
       </c>
     </row>
     <row r="5">
@@ -623,25 +623,25 @@
         <v>0.75</v>
       </c>
       <c r="E5" t="n">
-        <v>6038877197.75</v>
+        <v>11308668299.67</v>
       </c>
       <c r="F5" t="n">
-        <v>-800000000</v>
+        <v>-950368395.63</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>45291578.983125</v>
+        <v>84815012.24752501</v>
       </c>
       <c r="I5" t="n">
-        <v>-51291578.983125</v>
+        <v>-91942775.21474999</v>
       </c>
       <c r="J5" t="n">
-        <v>45291578.983125</v>
+        <v>84815012.24752501</v>
       </c>
       <c r="K5" t="n">
-        <v>-51291578.983125</v>
+        <v>-91942775.21474999</v>
       </c>
     </row>
     <row r="6">
@@ -662,25 +662,25 @@
         <v>0.6666666666666667</v>
       </c>
       <c r="E6" t="n">
-        <v>138537078.78</v>
+        <v>287898315.0900002</v>
       </c>
       <c r="F6" t="n">
-        <v>-800000000</v>
+        <v>-937266212.77</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>923580.5252</v>
+        <v>1919322.100600001</v>
       </c>
       <c r="I6" t="n">
-        <v>-6256913.858533333</v>
+        <v>-8167763.519066669</v>
       </c>
       <c r="J6" t="n">
-        <v>923580.5252</v>
+        <v>1919322.100600001</v>
       </c>
       <c r="K6" t="n">
-        <v>-6256913.858533333</v>
+        <v>-8167763.519066669</v>
       </c>
     </row>
     <row r="7">
@@ -701,25 +701,25 @@
         <v>0.5833333333333333</v>
       </c>
       <c r="E7" t="n">
-        <v>2293685276.16</v>
+        <v>4592568652.700001</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>-933556315.13</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>13379830.7776</v>
+        <v>26789983.80741667</v>
       </c>
       <c r="I7" t="n">
-        <v>-13379830.7776</v>
+        <v>-32235728.97900834</v>
       </c>
       <c r="J7" t="n">
-        <v>13379830.7776</v>
+        <v>26789983.80741667</v>
       </c>
       <c r="K7" t="n">
-        <v>-13379830.7776</v>
+        <v>-32235728.97900834</v>
       </c>
     </row>
     <row r="8">
@@ -740,25 +740,25 @@
         <v>0.5</v>
       </c>
       <c r="E8" t="n">
-        <v>6994820480.68</v>
+        <v>14895344121.75</v>
       </c>
       <c r="F8" t="n">
-        <v>-400000000</v>
+        <v>-534184986.24</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>34974102.4034</v>
+        <v>74476720.60875</v>
       </c>
       <c r="I8" t="n">
-        <v>-36974102.4034</v>
+        <v>-77147645.53995</v>
       </c>
       <c r="J8" t="n">
-        <v>34974102.4034</v>
+        <v>74476720.60875</v>
       </c>
       <c r="K8" t="n">
-        <v>-36974102.4034</v>
+        <v>-77147645.53995</v>
       </c>
     </row>
     <row r="9">
@@ -779,25 +779,25 @@
         <v>0.4166666666666666</v>
       </c>
       <c r="E9" t="n">
-        <v>-1132468695.5</v>
+        <v>-2265065811.22</v>
       </c>
       <c r="F9" t="n">
-        <v>-400000000</v>
+        <v>-522253278.41</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>-4718619.564583333</v>
+        <v>-9437774.213416666</v>
       </c>
       <c r="I9" t="n">
-        <v>3051952.897916666</v>
+        <v>7261718.886708331</v>
       </c>
       <c r="J9" t="n">
-        <v>-4718619.564583333</v>
+        <v>-9437774.213416666</v>
       </c>
       <c r="K9" t="n">
-        <v>3051952.897916666</v>
+        <v>7261718.886708331</v>
       </c>
     </row>
     <row r="10">
@@ -818,25 +818,25 @@
         <v>0.3333333333333334</v>
       </c>
       <c r="E10" t="n">
-        <v>-826591809.5599999</v>
+        <v>-1653631904.25</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>-512692413.08</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>-2755306.031866667</v>
+        <v>-5512106.347500001</v>
       </c>
       <c r="I10" t="n">
-        <v>2755306.031866667</v>
+        <v>3803131.637233334</v>
       </c>
       <c r="J10" t="n">
-        <v>-2755306.031866667</v>
+        <v>-5512106.347500001</v>
       </c>
       <c r="K10" t="n">
-        <v>2755306.031866667</v>
+        <v>3803131.637233334</v>
       </c>
     </row>
     <row r="11">
@@ -857,25 +857,25 @@
         <v>0.25</v>
       </c>
       <c r="E11" t="n">
-        <v>-479933073.1900001</v>
+        <v>-1103413874.16</v>
       </c>
       <c r="F11" t="n">
-        <v>-400000000</v>
+        <v>-522547792.53</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>-1199832.682975</v>
+        <v>-2758534.6854</v>
       </c>
       <c r="I11" t="n">
-        <v>199832.6829750001</v>
+        <v>1452165.204075</v>
       </c>
       <c r="J11" t="n">
-        <v>-1199832.682975</v>
+        <v>-2758534.6854</v>
       </c>
       <c r="K11" t="n">
-        <v>199832.6829750001</v>
+        <v>1452165.204075</v>
       </c>
     </row>
     <row r="12">
@@ -896,25 +896,25 @@
         <v>0.1666666666666666</v>
       </c>
       <c r="E12" t="n">
-        <v>-818538934.8799999</v>
+        <v>-1617508459.13</v>
       </c>
       <c r="F12" t="n">
-        <v>-400000000</v>
+        <v>-516937918.48</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>-1364231.558133333</v>
+        <v>-2695847.431883333</v>
       </c>
       <c r="I12" t="n">
-        <v>697564.8914666664</v>
+        <v>1834284.234416666</v>
       </c>
       <c r="J12" t="n">
-        <v>-1364231.558133333</v>
+        <v>-2695847.431883333</v>
       </c>
       <c r="K12" t="n">
-        <v>697564.8914666664</v>
+        <v>1834284.234416666</v>
       </c>
     </row>
     <row r="13">
@@ -935,25 +935,25 @@
         <v>0.08333333333333337</v>
       </c>
       <c r="E13" t="n">
-        <v>-811840769.16</v>
+        <v>-1623521087.52</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>-503998763.6</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>-676533.9743000002</v>
+        <v>-1352934.239600001</v>
       </c>
       <c r="I13" t="n">
-        <v>676533.9743000002</v>
+        <v>932935.2699333339</v>
       </c>
       <c r="J13" t="n">
-        <v>-676533.9743000002</v>
+        <v>-1352934.239600001</v>
       </c>
       <c r="K13" t="n">
-        <v>676533.9743000002</v>
+        <v>932935.2699333339</v>
       </c>
     </row>
     <row r="14">
@@ -974,10 +974,10 @@
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>-434460589.52</v>
+        <v>-1146624337.12</v>
       </c>
       <c r="F14" t="n">
-        <v>-400000000</v>
+        <v>-520727333.41</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
@@ -1058,25 +1058,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>17888722698.62</v>
+        <v>35574227907.64</v>
       </c>
       <c r="C2" t="n">
-        <v>-12800000000</v>
+        <v>-16354326135.91</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>133554358.2016317</v>
+        <v>265964192.380636</v>
       </c>
       <c r="F2" t="n">
-        <v>-240335180.1194399</v>
+        <v>-389561322.0670658</v>
       </c>
       <c r="G2" t="n">
-        <v>133554358.2016317</v>
+        <v>265964192.380636</v>
       </c>
       <c r="H2" t="n">
-        <v>-240335180.1194399</v>
+        <v>-389561322.0670658</v>
       </c>
     </row>
   </sheetData>
@@ -1132,13 +1132,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>-1635690752.42</v>
+        <v>-3271381504.99</v>
       </c>
       <c r="D2" t="n">
-        <v>-551041892.6027397</v>
+        <v>-1102083785.205479</v>
       </c>
       <c r="E2" t="n">
-        <v>-2186732645.02274</v>
+        <v>-4373465290.195479</v>
       </c>
     </row>
     <row r="3">
@@ -1153,13 +1153,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>891224973.27</v>
+        <v>1772042953.29</v>
       </c>
       <c r="D3" t="n">
-        <v>52385409.72</v>
+        <v>102556093.5293151</v>
       </c>
       <c r="E3" t="n">
-        <v>943610382.99</v>
+        <v>1874599046.819315</v>
       </c>
     </row>
     <row r="4">
@@ -1174,13 +1174,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1602040037.16</v>
+        <v>3196426808.51</v>
       </c>
       <c r="D4" t="n">
-        <v>168754858.2541759</v>
+        <v>337567414.8186869</v>
       </c>
       <c r="E4" t="n">
-        <v>1770794895.414176</v>
+        <v>3533994223.328687</v>
       </c>
     </row>
   </sheetData>
@@ -1226,13 +1226,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>857574258.01</v>
+        <v>1697088256.81</v>
       </c>
       <c r="C2" t="n">
-        <v>-329901624.6285638</v>
+        <v>-661960276.8574774</v>
       </c>
       <c r="D2" t="n">
-        <v>527672633.3814361</v>
+        <v>1035127979.952522</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix tenor bucketing: ceil -> round to correctly assign end-of-month flows
math.ceil mapped Jan 31 (31 days = 1.018M) to the 2M bucket instead of 1M.
Changing to max(1, round(...)) puts end-of-month flows in the correct bucket
(e.g. product 6000 1M, previously absent, now appears in ir_gap_beh_a).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/irrbb_calc/output/nii_results.xlsx
+++ b/irrbb_calc/output/nii_results.xlsx
@@ -545,25 +545,25 @@
         <v>0.9166666666666666</v>
       </c>
       <c r="E3" t="n">
-        <v>4214343154.54</v>
+        <v>16458155778.43</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>-948926786.59</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>38631478.91661666</v>
+        <v>150866427.9689417</v>
       </c>
       <c r="I3" t="n">
-        <v>-38631478.91661666</v>
+        <v>-159564923.5126833</v>
       </c>
       <c r="J3" t="n">
-        <v>38631478.91661666</v>
+        <v>150866427.9689417</v>
       </c>
       <c r="K3" t="n">
-        <v>-38631478.91661666</v>
+        <v>-159564923.5126833</v>
       </c>
     </row>
     <row r="4">
@@ -584,25 +584,25 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="E4" t="n">
-        <v>21654457449.59</v>
+        <v>9948663064.66</v>
       </c>
       <c r="F4" t="n">
-        <v>-1888284222.06</v>
+        <v>-939357435.47</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>180453812.0799167</v>
+        <v>82905525.53883334</v>
       </c>
       <c r="I4" t="n">
-        <v>-196189513.9304167</v>
+        <v>-90733504.16775</v>
       </c>
       <c r="J4" t="n">
-        <v>180453812.0799167</v>
+        <v>82905525.53883334</v>
       </c>
       <c r="K4" t="n">
-        <v>-196189513.9304167</v>
+        <v>-90733504.16775</v>
       </c>
     </row>
     <row r="5">
@@ -623,7 +623,7 @@
         <v>0.75</v>
       </c>
       <c r="E5" t="n">
-        <v>11308668299.67</v>
+        <v>11099174132.28</v>
       </c>
       <c r="F5" t="n">
         <v>-950368395.63</v>
@@ -632,16 +632,16 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>84815012.24752501</v>
+        <v>83243805.9921</v>
       </c>
       <c r="I5" t="n">
-        <v>-91942775.21474999</v>
+        <v>-90371568.95932499</v>
       </c>
       <c r="J5" t="n">
-        <v>84815012.24752501</v>
+        <v>83243805.9921</v>
       </c>
       <c r="K5" t="n">
-        <v>-91942775.21474999</v>
+        <v>-90371568.95932499</v>
       </c>
     </row>
     <row r="6">
@@ -662,7 +662,7 @@
         <v>0.6666666666666667</v>
       </c>
       <c r="E6" t="n">
-        <v>287898315.0900002</v>
+        <v>3589192236.5</v>
       </c>
       <c r="F6" t="n">
         <v>-937266212.77</v>
@@ -671,16 +671,16 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>1919322.100600001</v>
+        <v>23927948.24333334</v>
       </c>
       <c r="I6" t="n">
-        <v>-8167763.519066669</v>
+        <v>-30176389.6618</v>
       </c>
       <c r="J6" t="n">
-        <v>1919322.100600001</v>
+        <v>23927948.24333334</v>
       </c>
       <c r="K6" t="n">
-        <v>-8167763.519066669</v>
+        <v>-30176389.6618</v>
       </c>
     </row>
     <row r="7">
@@ -701,7 +701,7 @@
         <v>0.5833333333333333</v>
       </c>
       <c r="E7" t="n">
-        <v>4592568652.700001</v>
+        <v>1292202215.83</v>
       </c>
       <c r="F7" t="n">
         <v>-933556315.13</v>
@@ -710,16 +710,16 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>26789983.80741667</v>
+        <v>7537846.259008332</v>
       </c>
       <c r="I7" t="n">
-        <v>-32235728.97900834</v>
+        <v>-12983591.4306</v>
       </c>
       <c r="J7" t="n">
-        <v>26789983.80741667</v>
+        <v>7537846.259008332</v>
       </c>
       <c r="K7" t="n">
-        <v>-32235728.97900834</v>
+        <v>-12983591.4306</v>
       </c>
     </row>
     <row r="8">
@@ -740,7 +740,7 @@
         <v>0.5</v>
       </c>
       <c r="E8" t="n">
-        <v>14895344121.75</v>
+        <v>14731847447.54</v>
       </c>
       <c r="F8" t="n">
         <v>-534184986.24</v>
@@ -749,16 +749,16 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>74476720.60875</v>
+        <v>73659237.2377</v>
       </c>
       <c r="I8" t="n">
-        <v>-77147645.53995</v>
+        <v>-76330162.1689</v>
       </c>
       <c r="J8" t="n">
-        <v>74476720.60875</v>
+        <v>73659237.2377</v>
       </c>
       <c r="K8" t="n">
-        <v>-77147645.53995</v>
+        <v>-76330162.1689</v>
       </c>
     </row>
     <row r="9">
@@ -779,7 +779,7 @@
         <v>0.4166666666666666</v>
       </c>
       <c r="E9" t="n">
-        <v>-2265065811.22</v>
+        <v>-2289519782.09</v>
       </c>
       <c r="F9" t="n">
         <v>-522253278.41</v>
@@ -788,16 +788,16 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>-9437774.213416666</v>
+        <v>-9539665.758708332</v>
       </c>
       <c r="I9" t="n">
-        <v>7261718.886708331</v>
+        <v>7363610.431999998</v>
       </c>
       <c r="J9" t="n">
-        <v>-9437774.213416666</v>
+        <v>-9539665.758708332</v>
       </c>
       <c r="K9" t="n">
-        <v>7261718.886708331</v>
+        <v>7363610.431999998</v>
       </c>
     </row>
     <row r="10">
@@ -818,7 +818,7 @@
         <v>0.3333333333333334</v>
       </c>
       <c r="E10" t="n">
-        <v>-1653631904.25</v>
+        <v>-1632583477.45</v>
       </c>
       <c r="F10" t="n">
         <v>-512692413.08</v>
@@ -827,16 +827,16 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>-5512106.347500001</v>
+        <v>-5441944.924833334</v>
       </c>
       <c r="I10" t="n">
-        <v>3803131.637233334</v>
+        <v>3732970.214566668</v>
       </c>
       <c r="J10" t="n">
-        <v>-5512106.347500001</v>
+        <v>-5441944.924833334</v>
       </c>
       <c r="K10" t="n">
-        <v>3803131.637233334</v>
+        <v>3732970.214566668</v>
       </c>
     </row>
     <row r="11">
@@ -857,7 +857,7 @@
         <v>0.25</v>
       </c>
       <c r="E11" t="n">
-        <v>-1103413874.16</v>
+        <v>-1062307276.65</v>
       </c>
       <c r="F11" t="n">
         <v>-522547792.53</v>
@@ -866,16 +866,16 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>-2758534.6854</v>
+        <v>-2655768.191625</v>
       </c>
       <c r="I11" t="n">
-        <v>1452165.204075</v>
+        <v>1349398.7103</v>
       </c>
       <c r="J11" t="n">
-        <v>-2758534.6854</v>
+        <v>-2655768.191625</v>
       </c>
       <c r="K11" t="n">
-        <v>1452165.204075</v>
+        <v>1349398.7103</v>
       </c>
     </row>
     <row r="12">
@@ -896,7 +896,7 @@
         <v>0.1666666666666666</v>
       </c>
       <c r="E12" t="n">
-        <v>-1617508459.13</v>
+        <v>-1673310261.43</v>
       </c>
       <c r="F12" t="n">
         <v>-516937918.48</v>
@@ -905,16 +905,16 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>-2695847.431883333</v>
+        <v>-2788850.435716666</v>
       </c>
       <c r="I12" t="n">
-        <v>1834284.234416666</v>
+        <v>1927287.23825</v>
       </c>
       <c r="J12" t="n">
-        <v>-2695847.431883333</v>
+        <v>-2788850.435716666</v>
       </c>
       <c r="K12" t="n">
-        <v>1834284.234416666</v>
+        <v>1927287.23825</v>
       </c>
     </row>
     <row r="13">
@@ -935,7 +935,7 @@
         <v>0.08333333333333337</v>
       </c>
       <c r="E13" t="n">
-        <v>-1623521087.52</v>
+        <v>-1603690311.79</v>
       </c>
       <c r="F13" t="n">
         <v>-503998763.6</v>
@@ -944,16 +944,16 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>-1352934.239600001</v>
+        <v>-1336408.593158334</v>
       </c>
       <c r="I13" t="n">
-        <v>932935.2699333339</v>
+        <v>916409.6234916671</v>
       </c>
       <c r="J13" t="n">
-        <v>-1352934.239600001</v>
+        <v>-1336408.593158334</v>
       </c>
       <c r="K13" t="n">
-        <v>932935.2699333339</v>
+        <v>916409.6234916671</v>
       </c>
     </row>
     <row r="14">
@@ -974,7 +974,7 @@
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>-1146624337.12</v>
+        <v>-1067621671.08</v>
       </c>
       <c r="F14" t="n">
         <v>-520727333.41</v>
@@ -1058,7 +1058,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>35574227907.64</v>
+        <v>35820915482.45</v>
       </c>
       <c r="C2" t="n">
         <v>-16354326135.91</v>
@@ -1067,16 +1067,16 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>265964192.380636</v>
+        <v>281013212.8734859</v>
       </c>
       <c r="F2" t="n">
-        <v>-389561322.0670658</v>
+        <v>-405401114.8820741</v>
       </c>
       <c r="G2" t="n">
-        <v>265964192.380636</v>
+        <v>281013212.8734859</v>
       </c>
       <c r="H2" t="n">
-        <v>-389561322.0670658</v>
+        <v>-405401114.8820741</v>
       </c>
     </row>
   </sheetData>

</xml_diff>